<commit_message>
PR03 - Step 1.4.1 - Complete
Preprocess Population Data Done! Dumb spelling mistake on two of the features to drop.
</commit_message>
<xml_diff>
--- a/Project 03/identify_customer_segments/feature_selection.xlsx
+++ b/Project 03/identify_customer_segments/feature_selection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Udacity Nanodegrees\ud-ml-pytorch\Project 03\identify_customer_segments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504AB0D7-73B0-4418-AA4F-9EC85B548A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3254ED70-BAB6-49EA-B684-C7FE70BD7967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38295" yWindow="0" windowWidth="19350" windowHeight="20985" xr2:uid="{776CD450-A4BF-432C-A298-8B7F7D26585D}"/>
+    <workbookView xWindow="28680" yWindow="15825" windowWidth="14595" windowHeight="15960" xr2:uid="{776CD450-A4BF-432C-A298-8B7F7D26585D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="112">
   <si>
     <t>'AGER_TYP',</t>
   </si>
@@ -356,9 +356,6 @@
     <t>CATEGORICAL</t>
   </si>
   <si>
-    <t>NEW</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 'DECADE'</t>
   </si>
   <si>
@@ -369,6 +366,15 @@
   </si>
   <si>
     <t xml:space="preserve"> 'LIFE_STAGE'</t>
+  </si>
+  <si>
+    <t>COL OBTAINED FROM ENGINEERING</t>
+  </si>
+  <si>
+    <t>FINAL CHECK</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
@@ -418,7 +424,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -441,6 +447,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -456,13 +482,21 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -797,69 +831,74 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE12CC76-8952-4997-9B6A-52BC5030CAFF}">
-  <dimension ref="A1:I90"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:J90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" style="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.42578125" customWidth="1"/>
     <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="1:10" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="12"/>
+      <c r="B1" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F1" s="2" t="s">
+      <c r="E1" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="F1" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="12" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="14" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="5" t="s">
         <v>104</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="E2" s="5"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="10"/>
+      <c r="B3" s="1"/>
       <c r="C3" s="1" t="s">
         <v>100</v>
       </c>
@@ -877,12 +916,15 @@
       <c r="I3" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -902,12 +944,15 @@
       <c r="I4" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -925,14 +970,17 @@
         <v>6</v>
       </c>
       <c r="I5" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="J5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="10"/>
+      <c r="B6" s="1"/>
       <c r="C6" s="1" t="s">
         <v>100</v>
       </c>
@@ -950,12 +998,15 @@
       <c r="I6" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="10"/>
+      <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
         <v>100</v>
       </c>
@@ -973,12 +1024,15 @@
       <c r="I7" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="10"/>
+      <c r="B8" s="1"/>
       <c r="C8" s="1" t="s">
         <v>100</v>
       </c>
@@ -996,12 +1050,15 @@
       <c r="I8" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="10"/>
+      <c r="B9" s="1"/>
       <c r="C9" s="1" t="s">
         <v>100</v>
       </c>
@@ -1019,12 +1076,15 @@
       <c r="I9" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J9" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="10"/>
+      <c r="B10" s="1"/>
       <c r="C10" s="1" t="s">
         <v>100</v>
       </c>
@@ -1042,12 +1102,15 @@
       <c r="I10" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="10"/>
+      <c r="B11" s="1"/>
       <c r="C11" s="1" t="s">
         <v>100</v>
       </c>
@@ -1065,12 +1128,15 @@
       <c r="I11" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C12" s="1" t="s">
@@ -1090,12 +1156,15 @@
       <c r="I12" s="1">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J12" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="11"/>
+      <c r="B13" s="5"/>
       <c r="C13" s="5" t="s">
         <v>99</v>
       </c>
@@ -1112,11 +1181,11 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -1134,14 +1203,17 @@
         <v>12</v>
       </c>
       <c r="I14" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="J14" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="7" t="s">
         <v>104</v>
       </c>
       <c r="C15" s="7"/>
@@ -1154,11 +1226,11 @@
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="10"/>
+      <c r="B16" s="1"/>
       <c r="C16" s="1" t="s">
         <v>100</v>
       </c>
@@ -1176,12 +1248,15 @@
       <c r="I16" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="13"/>
+      <c r="B17" s="9"/>
       <c r="C17" s="9" t="s">
         <v>97</v>
       </c>
@@ -1198,11 +1273,11 @@
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="13"/>
+      <c r="B18" s="9"/>
       <c r="C18" s="9" t="s">
         <v>97</v>
       </c>
@@ -1219,11 +1294,11 @@
       <c r="H18" s="9"/>
       <c r="I18" s="9"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="7" t="s">
         <v>104</v>
       </c>
       <c r="C19" s="7"/>
@@ -1236,11 +1311,11 @@
       <c r="H19" s="7"/>
       <c r="I19" s="7"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -1258,14 +1333,17 @@
         <v>5</v>
       </c>
       <c r="I20" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="J20" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="7" t="s">
         <v>104</v>
       </c>
       <c r="C21" s="7"/>
@@ -1278,11 +1356,11 @@
       <c r="H21" s="7"/>
       <c r="I21" s="7"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C22" s="1" t="s">
@@ -1300,14 +1378,17 @@
         <v>5</v>
       </c>
       <c r="I22" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="J22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="7" t="s">
         <v>104</v>
       </c>
       <c r="C23" s="7"/>
@@ -1320,11 +1401,11 @@
       <c r="H23" s="7"/>
       <c r="I23" s="7"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="10"/>
+      <c r="B24" s="1"/>
       <c r="C24" s="1" t="s">
         <v>97</v>
       </c>
@@ -1340,14 +1421,14 @@
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="10"/>
+      <c r="B25" s="1"/>
       <c r="C25" s="1" t="s">
         <v>100</v>
       </c>
@@ -1365,12 +1446,15 @@
       <c r="I25" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J25" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="10"/>
+      <c r="B26" s="1"/>
       <c r="C26" s="1" t="s">
         <v>100</v>
       </c>
@@ -1388,12 +1472,15 @@
       <c r="I26" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J26" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="10"/>
+      <c r="B27" s="1"/>
       <c r="C27" s="1" t="s">
         <v>100</v>
       </c>
@@ -1411,12 +1498,15 @@
       <c r="I27" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J27" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="10"/>
+      <c r="B28" s="1"/>
       <c r="C28" s="1" t="s">
         <v>100</v>
       </c>
@@ -1434,12 +1524,15 @@
       <c r="I28" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J28" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="10"/>
+      <c r="B29" s="1"/>
       <c r="C29" s="1" t="s">
         <v>100</v>
       </c>
@@ -1457,12 +1550,15 @@
       <c r="I29" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J29" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="10"/>
+      <c r="B30" s="1"/>
       <c r="C30" s="1" t="s">
         <v>100</v>
       </c>
@@ -1480,12 +1576,15 @@
       <c r="I30" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J30" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="10"/>
+      <c r="B31" s="1"/>
       <c r="C31" s="1" t="s">
         <v>100</v>
       </c>
@@ -1503,12 +1602,15 @@
       <c r="I31" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J31" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B32" s="10"/>
+      <c r="B32" s="1"/>
       <c r="C32" s="1" t="s">
         <v>100</v>
       </c>
@@ -1526,12 +1628,15 @@
       <c r="I32" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J32" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B33" s="10"/>
+      <c r="B33" s="1"/>
       <c r="C33" s="1" t="s">
         <v>100</v>
       </c>
@@ -1549,12 +1654,15 @@
       <c r="I33" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J33" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="10"/>
+      <c r="B34" s="1"/>
       <c r="C34" s="1" t="s">
         <v>100</v>
       </c>
@@ -1572,12 +1680,15 @@
       <c r="I34" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J34" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="10"/>
+      <c r="B35" s="1"/>
       <c r="C35" s="1" t="s">
         <v>100</v>
       </c>
@@ -1595,12 +1706,15 @@
       <c r="I35" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J35" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B36" s="10"/>
+      <c r="B36" s="1"/>
       <c r="C36" s="1" t="s">
         <v>100</v>
       </c>
@@ -1618,12 +1732,15 @@
       <c r="I36" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J36" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="10"/>
+      <c r="B37" s="1"/>
       <c r="C37" s="1" t="s">
         <v>100</v>
       </c>
@@ -1641,12 +1758,15 @@
       <c r="I37" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J37" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="10"/>
+      <c r="B38" s="1"/>
       <c r="C38" s="1" t="s">
         <v>100</v>
       </c>
@@ -1664,12 +1784,15 @@
       <c r="I38" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J38" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="10"/>
+      <c r="B39" s="1"/>
       <c r="C39" s="1" t="s">
         <v>100</v>
       </c>
@@ -1687,12 +1810,15 @@
       <c r="I39" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J39" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B40" s="10" t="s">
+      <c r="B40" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C40" s="1" t="s">
@@ -1710,14 +1836,17 @@
         <v>4</v>
       </c>
       <c r="I40" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="J40" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="12" t="s">
+      <c r="B41" s="7" t="s">
         <v>104</v>
       </c>
       <c r="C41" s="7"/>
@@ -1730,11 +1859,11 @@
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="5" t="s">
         <v>104</v>
       </c>
       <c r="C42" s="5"/>
@@ -1747,11 +1876,11 @@
       <c r="H42" s="5"/>
       <c r="I42" s="5"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B43" s="10" t="s">
+      <c r="B43" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C43" s="1" t="s">
@@ -1771,12 +1900,15 @@
       <c r="I43" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J43" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B44" s="10" t="s">
+      <c r="B44" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C44" s="1" t="s">
@@ -1796,12 +1928,15 @@
       <c r="I44" s="1">
         <v>6</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J44" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B45" s="11"/>
+      <c r="B45" s="5"/>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
         <v>101</v>
@@ -1816,11 +1951,11 @@
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="10"/>
+      <c r="B46" s="1"/>
       <c r="C46" s="1" t="s">
         <v>99</v>
       </c>
@@ -1838,12 +1973,15 @@
       <c r="I46" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J46" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B47" s="10"/>
+      <c r="B47" s="1"/>
       <c r="C47" s="1" t="s">
         <v>99</v>
       </c>
@@ -1861,12 +1999,15 @@
       <c r="I47" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J47" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B48" s="10"/>
+      <c r="B48" s="1"/>
       <c r="C48" s="1" t="s">
         <v>100</v>
       </c>
@@ -1884,12 +2025,15 @@
       <c r="I48" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J48" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B49" s="11" t="s">
+      <c r="B49" s="5" t="s">
         <v>104</v>
       </c>
       <c r="C49" s="5"/>
@@ -1902,11 +2046,11 @@
       <c r="H49" s="5"/>
       <c r="I49" s="5"/>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="10"/>
+      <c r="B50" s="1"/>
       <c r="C50" s="1" t="s">
         <v>100</v>
       </c>
@@ -1924,12 +2068,15 @@
       <c r="I50" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J50" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B51" s="10"/>
+      <c r="B51" s="1"/>
       <c r="C51" s="1" t="s">
         <v>100</v>
       </c>
@@ -1947,12 +2094,15 @@
       <c r="I51" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J51" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B52" s="10"/>
+      <c r="B52" s="1"/>
       <c r="C52" s="1" t="s">
         <v>99</v>
       </c>
@@ -1970,12 +2120,15 @@
       <c r="I52" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J52" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B53" s="10"/>
+      <c r="B53" s="1"/>
       <c r="C53" s="1" t="s">
         <v>99</v>
       </c>
@@ -1993,12 +2146,15 @@
       <c r="I53" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J53" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B54" s="12" t="s">
+      <c r="B54" s="7" t="s">
         <v>104</v>
       </c>
       <c r="C54" s="7"/>
@@ -2011,11 +2167,11 @@
       <c r="H54" s="7"/>
       <c r="I54" s="7"/>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B55" s="10"/>
+      <c r="B55" s="1"/>
       <c r="C55" s="1" t="s">
         <v>100</v>
       </c>
@@ -2033,12 +2189,15 @@
       <c r="I55" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J55" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B56" s="10"/>
+      <c r="B56" s="1"/>
       <c r="C56" s="1" t="s">
         <v>99</v>
       </c>
@@ -2056,12 +2215,15 @@
       <c r="I56" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J56" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B57" s="10" t="s">
+      <c r="B57" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C57" s="1" t="s">
@@ -2070,10 +2232,10 @@
       <c r="D57" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E57" s="1"/>
-      <c r="F57" s="1" t="s">
+      <c r="E57" s="1" t="s">
         <v>92</v>
       </c>
+      <c r="F57" s="1"/>
       <c r="G57" s="1"/>
       <c r="H57" s="1">
         <v>2</v>
@@ -2081,12 +2243,15 @@
       <c r="I57" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J57" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B58" s="13"/>
+      <c r="B58" s="9"/>
       <c r="C58" s="9" t="s">
         <v>97</v>
       </c>
@@ -2103,11 +2268,11 @@
       <c r="H58" s="9"/>
       <c r="I58" s="9"/>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B59" s="10" t="s">
+      <c r="B59" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C59" s="1" t="s">
@@ -2125,14 +2290,17 @@
         <v>9</v>
       </c>
       <c r="I59" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="J59" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B60" s="12" t="s">
+      <c r="B60" s="7" t="s">
         <v>104</v>
       </c>
       <c r="C60" s="7"/>
@@ -2145,11 +2313,11 @@
       <c r="H60" s="7"/>
       <c r="I60" s="7"/>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B61" s="10"/>
+      <c r="B61" s="1"/>
       <c r="C61" s="1" t="s">
         <v>97</v>
       </c>
@@ -2165,14 +2333,14 @@
       </c>
       <c r="H61" s="1"/>
       <c r="I61" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B62" s="10"/>
+      <c r="B62" s="1"/>
       <c r="C62" s="1" t="s">
         <v>100</v>
       </c>
@@ -2190,12 +2358,15 @@
       <c r="I62" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J62" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B63" s="10"/>
+      <c r="B63" s="1"/>
       <c r="C63" s="1" t="s">
         <v>100</v>
       </c>
@@ -2213,12 +2384,15 @@
       <c r="I63" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J63" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B64" s="10"/>
+      <c r="B64" s="1"/>
       <c r="C64" s="1" t="s">
         <v>100</v>
       </c>
@@ -2236,12 +2410,15 @@
       <c r="I64" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J64" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B65" s="10"/>
+      <c r="B65" s="1"/>
       <c r="C65" s="1" t="s">
         <v>100</v>
       </c>
@@ -2259,12 +2436,15 @@
       <c r="I65" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J65" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B66" s="11"/>
+      <c r="B66" s="5"/>
       <c r="C66" s="5" t="s">
         <v>97</v>
       </c>
@@ -2281,11 +2461,11 @@
       <c r="H66" s="5"/>
       <c r="I66" s="5"/>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B67" s="10"/>
+      <c r="B67" s="1"/>
       <c r="C67" s="1" t="s">
         <v>100</v>
       </c>
@@ -2293,7 +2473,7 @@
         <v>90</v>
       </c>
       <c r="E67" s="1"/>
-      <c r="F67" s="15" t="s">
+      <c r="F67" s="1" t="s">
         <v>89</v>
       </c>
       <c r="G67" s="1" t="s">
@@ -2303,12 +2483,15 @@
       <c r="I67" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J67" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B68" s="10"/>
+      <c r="B68" s="1"/>
       <c r="C68" s="1" t="s">
         <v>100</v>
       </c>
@@ -2316,7 +2499,7 @@
         <v>90</v>
       </c>
       <c r="E68" s="1"/>
-      <c r="F68" s="15" t="s">
+      <c r="F68" s="1" t="s">
         <v>89</v>
       </c>
       <c r="G68" s="1" t="s">
@@ -2326,12 +2509,15 @@
       <c r="I68" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J68" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B69" s="10"/>
+      <c r="B69" s="1"/>
       <c r="C69" s="1" t="s">
         <v>100</v>
       </c>
@@ -2339,7 +2525,7 @@
         <v>90</v>
       </c>
       <c r="E69" s="1"/>
-      <c r="F69" s="15" t="s">
+      <c r="F69" s="1" t="s">
         <v>89</v>
       </c>
       <c r="G69" s="1" t="s">
@@ -2349,12 +2535,15 @@
       <c r="I69" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J69" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B70" s="10"/>
+      <c r="B70" s="1"/>
       <c r="C70" s="1" t="s">
         <v>100</v>
       </c>
@@ -2362,7 +2551,7 @@
         <v>90</v>
       </c>
       <c r="E70" s="1"/>
-      <c r="F70" s="15" t="s">
+      <c r="F70" s="1" t="s">
         <v>89</v>
       </c>
       <c r="G70" s="1" t="s">
@@ -2372,12 +2561,15 @@
       <c r="I70" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J70" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B71" s="10"/>
+      <c r="B71" s="1"/>
       <c r="C71" s="1" t="s">
         <v>100</v>
       </c>
@@ -2385,7 +2577,7 @@
         <v>90</v>
       </c>
       <c r="E71" s="1"/>
-      <c r="F71" s="15" t="s">
+      <c r="F71" s="1" t="s">
         <v>89</v>
       </c>
       <c r="G71" s="1" t="s">
@@ -2395,12 +2587,15 @@
       <c r="I71" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J71" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B72" s="10"/>
+      <c r="B72" s="1"/>
       <c r="C72" s="1" t="s">
         <v>100</v>
       </c>
@@ -2408,7 +2603,7 @@
         <v>90</v>
       </c>
       <c r="E72" s="1"/>
-      <c r="F72" s="15" t="s">
+      <c r="F72" s="1" t="s">
         <v>89</v>
       </c>
       <c r="G72" s="1" t="s">
@@ -2418,12 +2613,15 @@
       <c r="I72" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J72" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B73" s="10"/>
+      <c r="B73" s="1"/>
       <c r="C73" s="1" t="s">
         <v>100</v>
       </c>
@@ -2431,7 +2629,7 @@
         <v>90</v>
       </c>
       <c r="E73" s="1"/>
-      <c r="F73" s="15" t="s">
+      <c r="F73" s="1" t="s">
         <v>89</v>
       </c>
       <c r="G73" s="1" t="s">
@@ -2441,12 +2639,15 @@
       <c r="I73" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J73" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B74" s="10"/>
+      <c r="B74" s="1"/>
       <c r="C74" s="1" t="s">
         <v>100</v>
       </c>
@@ -2454,7 +2655,7 @@
         <v>90</v>
       </c>
       <c r="E74" s="1"/>
-      <c r="F74" s="15" t="s">
+      <c r="F74" s="1" t="s">
         <v>89</v>
       </c>
       <c r="G74" s="1" t="s">
@@ -2464,12 +2665,15 @@
       <c r="I74" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J74" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B75" s="10"/>
+      <c r="B75" s="1"/>
       <c r="C75" s="1" t="s">
         <v>100</v>
       </c>
@@ -2477,7 +2681,7 @@
         <v>90</v>
       </c>
       <c r="E75" s="1"/>
-      <c r="F75" s="15" t="s">
+      <c r="F75" s="1" t="s">
         <v>89</v>
       </c>
       <c r="G75" s="1" t="s">
@@ -2487,12 +2691,15 @@
       <c r="I75" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J75" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B76" s="10"/>
+      <c r="B76" s="1"/>
       <c r="C76" s="1" t="s">
         <v>99</v>
       </c>
@@ -2510,12 +2717,15 @@
       <c r="I76" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J76" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B77" s="10"/>
+      <c r="B77" s="1"/>
       <c r="C77" s="1" t="s">
         <v>100</v>
       </c>
@@ -2533,12 +2743,15 @@
       <c r="I77" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J77" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B78" s="10"/>
+      <c r="B78" s="1"/>
       <c r="C78" s="1" t="s">
         <v>100</v>
       </c>
@@ -2556,12 +2769,15 @@
       <c r="I78" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J78" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B79" s="10"/>
+      <c r="B79" s="1"/>
       <c r="C79" s="1" t="s">
         <v>100</v>
       </c>
@@ -2579,12 +2795,15 @@
       <c r="I79" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J79" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B80" s="10"/>
+      <c r="B80" s="1"/>
       <c r="C80" s="1" t="s">
         <v>100</v>
       </c>
@@ -2602,12 +2821,15 @@
       <c r="I80" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J80" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B81" s="13"/>
+      <c r="B81" s="9"/>
       <c r="C81" s="9" t="s">
         <v>97</v>
       </c>
@@ -2624,11 +2846,11 @@
       <c r="H81" s="9"/>
       <c r="I81" s="9"/>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B82" s="10"/>
+      <c r="B82" s="1"/>
       <c r="C82" s="1" t="s">
         <v>100</v>
       </c>
@@ -2646,12 +2868,15 @@
       <c r="I82" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J82" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B83" s="10"/>
+      <c r="B83" s="1"/>
       <c r="C83" s="1" t="s">
         <v>100</v>
       </c>
@@ -2669,12 +2894,15 @@
       <c r="I83" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J83" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B84" s="10"/>
+      <c r="B84" s="1"/>
       <c r="C84" s="1" t="s">
         <v>100</v>
       </c>
@@ -2692,12 +2920,15 @@
       <c r="I84" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J84" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B85" s="10"/>
+      <c r="B85" s="1"/>
       <c r="C85" s="1" t="s">
         <v>100</v>
       </c>
@@ -2715,12 +2946,15 @@
       <c r="I85" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J85" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B86" s="10"/>
+      <c r="B86" s="1"/>
       <c r="C86" s="1" t="s">
         <v>100</v>
       </c>
@@ -2738,19 +2972,24 @@
       <c r="I86" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A87" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="B87" s="10"/>
+      <c r="J86" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A87" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="B87" s="1"/>
       <c r="C87" s="1" t="s">
         <v>102</v>
       </c>
       <c r="D87" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E87" s="1"/>
+      <c r="E87" s="1" t="s">
+        <v>92</v>
+      </c>
       <c r="F87" s="1" t="s">
         <v>89</v>
       </c>
@@ -2761,19 +3000,24 @@
       <c r="I87" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J87" s="15" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B88" s="10"/>
+        <v>106</v>
+      </c>
+      <c r="B88" s="1"/>
       <c r="C88" s="1" t="s">
         <v>88</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E88" s="1"/>
+      <c r="E88" s="1" t="s">
+        <v>92</v>
+      </c>
       <c r="F88" s="1" t="s">
         <v>89</v>
       </c>
@@ -2784,19 +3028,24 @@
       <c r="I88" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J88" s="15" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B89" s="10"/>
+        <v>107</v>
+      </c>
+      <c r="B89" s="1"/>
       <c r="C89" s="1" t="s">
         <v>100</v>
       </c>
       <c r="D89" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E89" s="1"/>
+      <c r="E89" s="1" t="s">
+        <v>92</v>
+      </c>
       <c r="F89" s="1" t="s">
         <v>89</v>
       </c>
@@ -2807,19 +3056,24 @@
       <c r="I89" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J89" s="15" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B90" s="10"/>
+        <v>108</v>
+      </c>
+      <c r="B90" s="1"/>
       <c r="C90" s="1" t="s">
         <v>100</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E90" s="1"/>
+      <c r="E90" s="1" t="s">
+        <v>92</v>
+      </c>
       <c r="F90" s="1" t="s">
         <v>89</v>
       </c>
@@ -2830,9 +3084,18 @@
       <c r="I90" s="1">
         <v>1</v>
       </c>
+      <c r="J90" s="16" t="s">
+        <v>111</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I90" xr:uid="{AE12CC76-8952-4997-9B6A-52BC5030CAFF}"/>
+  <autoFilter ref="A1:I90" xr:uid="{AE12CC76-8952-4997-9B6A-52BC5030CAFF}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="KEEP"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
PR03N - Fixed Up to Step 1.3
</commit_message>
<xml_diff>
--- a/Project 03/identify_customer_segments/feature_selection.xlsx
+++ b/Project 03/identify_customer_segments/feature_selection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Udacity Nanodegrees\ud-ml-pytorch\Project 03\identify_customer_segments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3254ED70-BAB6-49EA-B684-C7FE70BD7967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50310CDE-FD8D-4B1E-986D-B47717891C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="15825" windowWidth="14595" windowHeight="15960" xr2:uid="{776CD450-A4BF-432C-A298-8B7F7D26585D}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$98</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="120">
   <si>
     <t>'AGER_TYP',</t>
   </si>
@@ -375,6 +375,30 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'LP_LIFE_STAGE'</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'LP_INCOME_LEVEL'</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'LP_IS_INDEPENTENT'</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'LP_AGE_CLASS'</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'LP_IS_HOMEOWNER'</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'WOHN_NEIGHBORHOOD_Q'</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ' WOHN_IS_RURAL'</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'WHON_NEW_BUILDING'</t>
   </si>
 </sst>
 </file>
@@ -398,7 +422,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -407,19 +431,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
+        <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -471,32 +489,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -832,14 +849,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE12CC76-8952-4997-9B6A-52BC5030CAFF}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J90"/>
+  <dimension ref="A1:J98"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.42578125" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" customWidth="1"/>
     <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -848,32 +865,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12"/>
-      <c r="B1" s="12" t="s">
+      <c r="A1" s="7"/>
+      <c r="B1" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="J1" s="9" t="s">
         <v>110</v>
       </c>
     </row>
@@ -888,13 +905,13 @@
       <c r="D2" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="E2" s="11"/>
+      <c r="E2" s="15"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -920,7 +937,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -948,7 +965,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -976,7 +993,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -1002,7 +1019,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -1028,7 +1045,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -1054,7 +1071,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -1080,7 +1097,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -1106,7 +1123,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -1132,7 +1149,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -1181,28 +1198,28 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1" t="s">
+      <c r="D14" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1">
+      <c r="G14" s="13"/>
+      <c r="H14" s="13">
         <v>12</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="13">
         <v>13</v>
       </c>
       <c r="J14" t="s">
@@ -1210,196 +1227,216 @@
       </c>
     </row>
     <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7" t="s">
+      <c r="C15" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13">
+        <v>1</v>
+      </c>
+      <c r="J16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+    </row>
+    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1">
-        <v>1</v>
-      </c>
-      <c r="J16" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="D17" s="9" t="s">
+      <c r="E18" s="5"/>
+      <c r="F18" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+    </row>
+    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13">
+        <v>11</v>
+      </c>
+      <c r="I19" s="13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-    </row>
-    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="D18" s="9" t="s">
+      <c r="E20" s="13"/>
+      <c r="F20" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13">
+        <v>5</v>
+      </c>
+      <c r="I20" s="13">
+        <v>6</v>
+      </c>
+      <c r="J20" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13">
+        <v>10</v>
+      </c>
+      <c r="I21" s="13">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D22" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-    </row>
-    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19" s="7" t="s">
+      <c r="E22" s="13"/>
+      <c r="F22" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13">
+        <v>5</v>
+      </c>
+      <c r="I22" s="13">
+        <v>6</v>
+      </c>
+      <c r="J22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7" t="s">
+      <c r="C23" s="13"/>
+      <c r="D23" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1">
-        <v>5</v>
-      </c>
-      <c r="I20" s="1">
-        <v>6</v>
-      </c>
-      <c r="J20" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1">
-        <v>5</v>
-      </c>
-      <c r="I22" s="1">
-        <v>6</v>
-      </c>
-      <c r="J22" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
@@ -1420,11 +1457,9 @@
         <v>92</v>
       </c>
       <c r="H24" s="1"/>
-      <c r="I24" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I24" s="1"/>
+    </row>
+    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -1450,7 +1485,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -1476,7 +1511,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -1502,7 +1537,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -1528,7 +1563,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -1554,7 +1589,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -1580,7 +1615,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -1606,7 +1641,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -1632,7 +1667,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
@@ -1658,7 +1693,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -1684,7 +1719,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
@@ -1710,7 +1745,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
@@ -1736,7 +1771,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
@@ -1762,7 +1797,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
@@ -1788,7 +1823,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
@@ -1814,7 +1849,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
@@ -1843,40 +1878,40 @@
       </c>
     </row>
     <row r="41" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
+      <c r="A41" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="C41" s="7"/>
-      <c r="D41" s="7" t="s">
+      <c r="C41" s="13"/>
+      <c r="D41" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="E41" s="7"/>
-      <c r="F41" s="7"/>
-      <c r="G41" s="7"/>
-      <c r="H41" s="7"/>
-      <c r="I41" s="7"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="13"/>
+      <c r="I41" s="13"/>
     </row>
     <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="C42" s="5"/>
-      <c r="D42" s="5" t="s">
+      <c r="C42" s="13"/>
+      <c r="D42" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-      <c r="I42" s="5"/>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E42" s="13"/>
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
+      <c r="H42" s="13"/>
+      <c r="I42" s="13"/>
+    </row>
+    <row r="43" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
@@ -1904,7 +1939,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
@@ -1933,25 +1968,25 @@
       </c>
     </row>
     <row r="45" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="4" t="s">
+      <c r="A45" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B45" s="5"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5" t="s">
+      <c r="B45" s="13"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="E45" s="5"/>
-      <c r="F45" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="G45" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="H45" s="5"/>
-      <c r="I45" s="5"/>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E45" s="13"/>
+      <c r="F45" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="G45" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="H45" s="13"/>
+      <c r="I45" s="13"/>
+    </row>
+    <row r="46" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
@@ -1977,7 +2012,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
@@ -2003,7 +2038,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
@@ -2030,23 +2065,23 @@
       </c>
     </row>
     <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5" t="s">
+      <c r="C49" s="13"/>
+      <c r="D49" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
-      <c r="H49" s="5"/>
-      <c r="I49" s="5"/>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
+      <c r="H49" s="13"/>
+      <c r="I49" s="13"/>
+    </row>
+    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
@@ -2072,7 +2107,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
@@ -2098,7 +2133,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
@@ -2124,7 +2159,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
@@ -2151,23 +2186,31 @@
       </c>
     </row>
     <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B54" s="7" t="s">
+      <c r="B54" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="C54" s="7"/>
-      <c r="D54" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="E54" s="7"/>
-      <c r="F54" s="7"/>
-      <c r="G54" s="7"/>
-      <c r="H54" s="7"/>
-      <c r="I54" s="7"/>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C54" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D54" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E54" s="13"/>
+      <c r="F54" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G54" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="H54" s="13"/>
+      <c r="I54" s="13">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -2193,7 +2236,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
@@ -2219,7 +2262,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
@@ -2233,9 +2276,11 @@
         <v>90</v>
       </c>
       <c r="E57" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="F57" s="1"/>
       <c r="G57" s="1"/>
       <c r="H57" s="1">
         <v>2</v>
@@ -2247,28 +2292,28 @@
         <v>111</v>
       </c>
     </row>
-    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="8" t="s">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9" t="s">
+      <c r="B58" s="13"/>
+      <c r="C58" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="D58" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="E58" s="9"/>
-      <c r="F58" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="G58" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="H58" s="9"/>
-      <c r="I58" s="9"/>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D58" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E58" s="13"/>
+      <c r="F58" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="G58" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="H58" s="13"/>
+      <c r="I58" s="13"/>
+    </row>
+    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
@@ -2279,7 +2324,7 @@
         <v>91</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="E59" s="1"/>
       <c r="F59" s="1" t="s">
@@ -2289,29 +2334,37 @@
       <c r="H59" s="1">
         <v>9</v>
       </c>
-      <c r="I59" s="1">
-        <v>10</v>
-      </c>
+      <c r="I59" s="1"/>
       <c r="J59" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="6" t="s">
+      <c r="A60" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B60" s="7" t="s">
+      <c r="B60" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="C60" s="7"/>
-      <c r="D60" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="E60" s="7"/>
-      <c r="F60" s="7"/>
-      <c r="G60" s="7"/>
-      <c r="H60" s="7"/>
-      <c r="I60" s="7"/>
+      <c r="C60" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D60" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E60" s="13"/>
+      <c r="F60" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="G60" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="H60" s="13">
+        <v>44</v>
+      </c>
+      <c r="I60" s="13">
+        <v>45</v>
+      </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
@@ -2332,11 +2385,9 @@
         <v>92</v>
       </c>
       <c r="H61" s="1"/>
-      <c r="I61" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I61" s="1"/>
+    </row>
+    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>60</v>
       </c>
@@ -2362,7 +2413,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>61</v>
       </c>
@@ -2388,7 +2439,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>62</v>
       </c>
@@ -2414,7 +2465,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>63</v>
       </c>
@@ -2445,9 +2496,7 @@
         <v>64</v>
       </c>
       <c r="B66" s="5"/>
-      <c r="C66" s="5" t="s">
-        <v>97</v>
-      </c>
+      <c r="C66" s="5"/>
       <c r="D66" s="5" t="s">
         <v>101</v>
       </c>
@@ -2461,7 +2510,7 @@
       <c r="H66" s="5"/>
       <c r="I66" s="5"/>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>65</v>
       </c>
@@ -2487,7 +2536,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>66</v>
       </c>
@@ -2513,7 +2562,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>67</v>
       </c>
@@ -2539,7 +2588,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>68</v>
       </c>
@@ -2565,7 +2614,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>69</v>
       </c>
@@ -2591,7 +2640,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>70</v>
       </c>
@@ -2617,7 +2666,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>71</v>
       </c>
@@ -2643,7 +2692,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>72</v>
       </c>
@@ -2669,7 +2718,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>73</v>
       </c>
@@ -2695,7 +2744,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>74</v>
       </c>
@@ -2721,7 +2770,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>75</v>
       </c>
@@ -2747,7 +2796,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>76</v>
       </c>
@@ -2773,7 +2822,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>77</v>
       </c>
@@ -2799,7 +2848,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>78</v>
       </c>
@@ -2826,27 +2875,27 @@
       </c>
     </row>
     <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="8" t="s">
+      <c r="A81" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B81" s="9"/>
-      <c r="C81" s="9" t="s">
+      <c r="B81" s="5"/>
+      <c r="C81" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="D81" s="9" t="s">
+      <c r="D81" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="E81" s="9"/>
-      <c r="F81" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="G81" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="H81" s="9"/>
-      <c r="I81" s="9"/>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E81" s="5"/>
+      <c r="F81" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G81" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H81" s="5"/>
+      <c r="I81" s="5"/>
+    </row>
+    <row r="82" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>80</v>
       </c>
@@ -2872,7 +2921,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>81</v>
       </c>
@@ -2898,7 +2947,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>82</v>
       </c>
@@ -2924,7 +2973,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>83</v>
       </c>
@@ -2950,7 +2999,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>84</v>
       </c>
@@ -2976,8 +3025,8 @@
         <v>111</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A87" s="10" t="s">
+    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="6" t="s">
         <v>105</v>
       </c>
       <c r="B87" s="1"/>
@@ -3000,11 +3049,11 @@
       <c r="I87" s="1">
         <v>1</v>
       </c>
-      <c r="J87" s="15" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J87" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>106</v>
       </c>
@@ -3028,11 +3077,11 @@
       <c r="I88" s="1">
         <v>1</v>
       </c>
-      <c r="J88" s="15" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J88" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>107</v>
       </c>
@@ -3056,11 +3105,11 @@
       <c r="I89" s="1">
         <v>1</v>
       </c>
-      <c r="J89" s="15" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J89" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>108</v>
       </c>
@@ -3084,12 +3133,221 @@
       <c r="I90" s="1">
         <v>1</v>
       </c>
-      <c r="J90" s="16" t="s">
-        <v>111</v>
+      <c r="J90" s="11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C91" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D91" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H91" s="1">
+        <v>5</v>
+      </c>
+      <c r="I91" s="14">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B92" s="1"/>
+      <c r="C92" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H92" s="1"/>
+      <c r="I92" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B93" s="1"/>
+      <c r="C93" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H93" s="1"/>
+      <c r="I93" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B94" s="1"/>
+      <c r="C94" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H94" s="1"/>
+      <c r="I94" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B95" s="1"/>
+      <c r="C95" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G95" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H95" s="1"/>
+      <c r="I95" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B96" s="1"/>
+      <c r="C96" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="D96" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E96" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="F96" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G96" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="H96" s="1"/>
+      <c r="I96" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B97" s="1"/>
+      <c r="C97" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D97" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E97" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="F97" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G97" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="H97" s="1"/>
+      <c r="I97" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B98" s="1"/>
+      <c r="C98" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D98" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E98" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="F98" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G98" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="H98" s="1"/>
+      <c r="I98" s="1">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I90" xr:uid="{AE12CC76-8952-4997-9B6A-52BC5030CAFF}">
+  <autoFilter ref="A1:I98" xr:uid="{AE12CC76-8952-4997-9B6A-52BC5030CAFF}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="MIXED"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="3">
       <filters>
         <filter val="KEEP"/>

</xml_diff>